<commit_message>
Adiciona versão em PDF da planilha de atualização do débito
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RSEcSvs1Px517d8mUYokdi
</commit_message>
<xml_diff>
--- a/0800122-42.2025 - Francisca Sousa/Calculo atualizado - Francisca x Banco Pan.xlsx
+++ b/0800122-42.2025 - Francisca Sousa/Calculo atualizado - Francisca x Banco Pan.xlsx
@@ -979,7 +979,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1410,12 +1410,12 @@
       <c r="C47" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;CProc. 0800122-42.2025.8.18.0061 – &amp;A – pág. &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
@@ -1424,7 +1424,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1688,12 +1688,12 @@
       <c r="F16" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;CProc. 0800122-42.2025.8.18.0061 – &amp;A – pág. &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
@@ -1702,7 +1702,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2388,12 +2388,12 @@
       <c r="E45" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;CProc. 0800122-42.2025.8.18.0061 – &amp;A – pág. &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>